<commit_message>
Shade claim rows by Claim Status in all workbooks
Adds row-level conditional formatting on every claim sheet (Master and
all six monthly files) keyed on column A. Rows with no Claim Status are
left unchanged. A colour legend is added to each Read Me tab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 00 Master.xlsx
+++ b/SPC26S1 - 00 Master.xlsx
@@ -3504,7 +3504,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="23">
     <dxf>
       <font>
         <color rgb="FF1F4E79"/>
@@ -3655,6 +3655,62 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD9D2E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE4A0C8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBFBFBF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -11696,7 +11752,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E79"/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="118" customWidth="1"/>
@@ -11853,7 +11909,127 @@
         <v>25</v>
       </c>
     </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="2"/>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Row colours by Claim Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="45" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each claim row is shaded by its Claim Status (column A) using conditional formatting, so the colour follows the status automatically when it is changed. Rows with no Claim Status keep their normal formatting. The deadline countdown columns keep their own colour bands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    PAID - green</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Finalized - blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Received - lavender</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Pending - yellow</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Under Review - orange</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Denied - red</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Rejected - pink</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Not found - grey</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Any other status is left unshaded.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A37">
+    <cfRule type="expression" dxfId="15" priority="1">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A38">
+    <cfRule type="expression" dxfId="16" priority="2">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A39">
+    <cfRule type="expression" dxfId="17" priority="3">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A40">
+    <cfRule type="expression" dxfId="18" priority="4">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A41">
+    <cfRule type="expression" dxfId="19" priority="5">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A42">
+    <cfRule type="expression" dxfId="20" priority="6">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A43">
+    <cfRule type="expression" dxfId="21" priority="7">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A44">
+    <cfRule type="expression" dxfId="22" priority="8">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -69486,6 +69662,32 @@
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A2:AO1000">
+    <cfRule type="expression" dxfId="15" priority="16">
+      <formula>TRIM($A2)="PAID"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="17">
+      <formula>TRIM($A2)="Finalized"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="17" priority="18">
+      <formula>TRIM($A2)="Received"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="19">
+      <formula>TRIM($A2)="Pending"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="20">
+      <formula>TRIM($A2)="Under Review"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="21">
+      <formula>TRIM($A2)="Denied"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="22">
+      <formula>TRIM($A2)="Rejected"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="23">
+      <formula>TRIM($A2)="Not found"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Set Gold Kidney Health Plan claim 549178846 to Under Review
Claim Status and Notes on January ORTHO now match the other Gold Kidney
claims ('Under Review' / 'Waiting for account to get activated again').
The master's cached values are updated to match, and 'Under Review' is
added to January's status drop-down and Read Me status list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 00 Master.xlsx
+++ b/SPC26S1 - 00 Master.xlsx
@@ -4345,8 +4345,12 @@
           <cell r="K8"/>
         </row>
         <row r="9">
-          <cell r="A9"/>
-          <cell r="B9"/>
+          <cell r="A9" t="str">
+            <v>Under Review</v>
+          </cell>
+          <cell r="B9" t="str">
+            <v>Waiting for account to get activated again</v>
+          </cell>
           <cell r="C9">
             <v>46111</v>
           </cell>
@@ -66134,11 +66138,11 @@
     <row r="450" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A450" s="5" t="str">
         <f>IFERROR(IF(INDEX([1]ORTHO!$A$2:$A$10,MATCH($D450,[1]ORTHO!$D$2:$D$10,0))="","",INDEX([1]ORTHO!$A$2:$A$10,MATCH($D450,[1]ORTHO!$D$2:$D$10,0))),"")</f>
-        <v/>
+        <v>Under Review</v>
       </c>
       <c r="B450" s="5" t="str">
         <f>IFERROR(IF(INDEX([1]ORTHO!$B$2:$B$10,MATCH($D450,[1]ORTHO!$D$2:$D$10,0))="","",INDEX([1]ORTHO!$B$2:$B$10,MATCH($D450,[1]ORTHO!$D$2:$D$10,0))),"")</f>
-        <v/>
+        <v>Waiting for account to get activated again</v>
       </c>
       <c r="C450" s="6">
         <f>IFERROR(IF(INDEX([1]ORTHO!$C$2:$C$10,MATCH($D450,[1]ORTHO!$D$2:$D$10,0))="","",INDEX([1]ORTHO!$C$2:$C$10,MATCH($D450,[1]ORTHO!$D$2:$D$10,0))),"")</f>

</xml_diff>